<commit_message>
added floating action button for new product and validation on popup modal
</commit_message>
<xml_diff>
--- a/ReportsAndDocuments/presentation Qs.xlsx
+++ b/ReportsAndDocuments/presentation Qs.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\300392759\Downloads\Dev1\W26_4495_S3_ManeeshaE\ReportsAndDocuments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F479F4F-F3FF-444A-BD35-C23C4F62C6CA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99D4598B-021B-434B-9B12-388BA52C1234}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,9 +28,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1" uniqueCount="1">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
     <t>product category:added</t>
+  </si>
+  <si>
+    <t>fault:no admin pannel</t>
+  </si>
+  <si>
+    <t xml:space="preserve">error msg </t>
+  </si>
+  <si>
+    <t>appear on modal</t>
   </si>
 </sst>
 </file>
@@ -348,12 +357,25 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:B5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>2</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
final report changes to the proposal
</commit_message>
<xml_diff>
--- a/ReportsAndDocuments/presentation Qs.xlsx
+++ b/ReportsAndDocuments/presentation Qs.xlsx
@@ -5,15 +5,16 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\300392759\Downloads\Dev1\W26_4495_S3_ManeeshaE\ReportsAndDocuments\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\300392759\Downloads\dev3\W26_4495_S3_ManeeshaE\ReportsAndDocuments\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4C4F79BC-47D7-466E-808E-E918EB7F8FBF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97794B54-8DEF-40A0-A41B-84BB43D930C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet2" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -28,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="70" uniqueCount="31">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="139" uniqueCount="83">
   <si>
     <t>product category:added</t>
   </si>
@@ -121,13 +122,169 @@
   </si>
   <si>
     <t>change dropdown menu with modern menu options</t>
+  </si>
+  <si>
+    <t>Change Area</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Justification</t>
+  </si>
+  <si>
+    <t>Forecast Model</t>
+  </si>
+  <si>
+    <t>The SSA model provides more accurate, data‑driven, and scalable demand forecasts by analyzing historical time‑series data, enabling better production planning and dispatch decisions.</t>
+  </si>
+  <si>
+    <t>Forecasting Integration (New Addition)</t>
+  </si>
+  <si>
+    <t>ML‑based demand forecasting was fully embedded into the operational workflow and used as a core input for vendor recommendations.</t>
+  </si>
+  <si>
+    <t>Integrating forecasting directly into decision support improved system intelligence and ensured that recommendations were driven by future demand rather than static historical data.</t>
+  </si>
+  <si>
+    <t>Dashboard Architecture</t>
+  </si>
+  <si>
+    <t>The dashboard was upgraded from a static UI design to a fully dynamic, API‑driven architecture supporting real‑time data updates.</t>
+  </si>
+  <si>
+    <t>This change improved system responsiveness and enabled real‑time visibility of inventory, requests, forecasts, and recommendations, enhancing user decision‑making.</t>
+  </si>
+  <si>
+    <t>Authentication and Security</t>
+  </si>
+  <si>
+    <t>Role‑based authentication was implemented using ASP.NET Identity with JWT‑based authorization.</t>
+  </si>
+  <si>
+    <t>Secure role separation was required to protect sensitive data and enforce access control between farmer and vendor functionalities.</t>
+  </si>
+  <si>
+    <t>Recommendation Logic</t>
+  </si>
+  <si>
+    <t>The original optimization‑based approach was simplified into a weighted scoring‑based recommendation system.</t>
+  </si>
+  <si>
+    <t>The scoring approach improved interpretability and usability, making recommendation logic easier for non‑technical agricultural users to understand and trust.</t>
+  </si>
+  <si>
+    <t>Relationship Tracking Enhancement</t>
+  </si>
+  <si>
+    <t>A new relationship‑tracking entity was introduced to record historical farmer–vendor interactions and compute a relationship score.</t>
+  </si>
+  <si>
+    <t>Including relationship history improved recommendation accuracy by accounting for prior collaboration performance and trust.</t>
+  </si>
+  <si>
+    <t>Location Feature</t>
+  </si>
+  <si>
+    <t>Latitude and longitude fields were added to user profiles to support geospatial calculations.</t>
+  </si>
+  <si>
+    <t>Geolocation data is required to compute distances between farmers and vendors, which is essential for distance‑based ranking and logistics optimization.</t>
+  </si>
+  <si>
+    <t>Data Generation Strategy</t>
+  </si>
+  <si>
+    <t>The initial simulated dataset approach was enhanced to include multi‑period historical demand, inventory, and dispatch data.</t>
+  </si>
+  <si>
+    <t>More realistic historical data was necessary to support reliable machine learning forecasting and to reflect real‑world agricultural scenarios.</t>
+  </si>
+  <si>
+    <t>User Experience Improvements</t>
+  </si>
+  <si>
+    <t>Searchable dropdowns, improved navigation through a shared sidebar layout, and improved input validation were introduced.</t>
+  </si>
+  <si>
+    <t>These changes significantly improved usability, reduced user errors, and enhanced overall interaction efficiency for both farmer and vendor roles.</t>
+  </si>
+  <si>
+    <t>Chat Module</t>
+  </si>
+  <si>
+    <t>A real‑time communication module was added using SignalR.</t>
+  </si>
+  <si>
+    <t>Real‑time messaging was required to support timely coordination, negotiations, and clarification during dispatch and fulfillment processes.</t>
+  </si>
+  <si>
+    <t>The initially proposed simple logic‑based demand estimation approach and Moving Average algorithm was replaced with a machine learning‑based forecasting model using ML.NET Singular Spectrum Analysis (SSA).</t>
+  </si>
+  <si>
+    <t>The initially proposed simple logic-based demand estimation approach and Moving Average algorithm was replaced with a machine learning-based forecasting model using ML.NET Singular Spectrum Analysis (SSA).</t>
+  </si>
+  <si>
+    <t>The SSA model provides more accurate, data-driven, and scalable demand forecasts by analyzing historical time-series data, enabling better production planning and dispatch decisions.</t>
+  </si>
+  <si>
+    <t>ML-based demand forecasting was fully embedded into the operational workflow and used as a core input for vendor recommendations.</t>
+  </si>
+  <si>
+    <t>The dashboard was upgraded from a static UI design to a fully dynamic, API-driven architecture supporting real-time data updates.</t>
+  </si>
+  <si>
+    <t>This change improved system responsiveness and enabled real-time visibility of inventory, requests, forecasts, and recommendations, enhancing user decision-making.</t>
+  </si>
+  <si>
+    <t>Role-based authentication was implemented using ASP.NET Identity with JWT-based authorization.</t>
+  </si>
+  <si>
+    <t>The original optimization-based approach was simplified into a weighted scoring-based recommendation system.</t>
+  </si>
+  <si>
+    <t>The scoring approach improved interpretability and usability, making recommendation logic easier for non-technical agricultural users to understand and trust.</t>
+  </si>
+  <si>
+    <t>A new relationship-tracking entity was introduced to record historical farmer–vendor interactions and compute a relationship score.</t>
+  </si>
+  <si>
+    <t>Geolocation data is required to compute distances between farmers and vendors, which is essential for distance-based ranking and logistics optimization.</t>
+  </si>
+  <si>
+    <t>The initial simulated dataset approach was enhanced to include multi-period historical demand, inventory, and dispatch data.</t>
+  </si>
+  <si>
+    <t>More realistic historical data was necessary to support reliable machine learning forecasting and to reflect real-world agricultural scenarios.</t>
+  </si>
+  <si>
+    <t>Searchable dropdowns, improved navigation through a shared sidebar layout, hover-based details, and enhanced input validation were introduced.</t>
+  </si>
+  <si>
+    <t>A real-time communication module was added using SignalR.</t>
+  </si>
+  <si>
+    <t>Real-time messaging was required to support timely coordination, negotiations, and clarification during dispatch and fulfillment processes.</t>
+  </si>
+  <si>
+    <t>Image Integration (Unsplash API – New Addition)</t>
+  </si>
+  <si>
+    <t>Product images were integrated using the Unsplash API to dynamically display images in dropdowns and dashboards.</t>
+  </si>
+  <si>
+    <t>This enhancement improves visual clarity, user engagement, and usability. It eliminates the need for manual image uploads while providing high-quality, scalable visual content for better product identification.</t>
+  </si>
+  <si>
+    <t>Forecasting Integration</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -135,8 +292,29 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Segoe UI"/>
+      <family val="2"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -149,8 +327,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFF5F5F5"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -158,13 +342,46 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFE6E6E6"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFE6E6E6"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFE6E6E6"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFE6E6E6"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -740,4 +957,274 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{12F6663D-199B-475F-BB8E-399E72315137}">
+  <dimension ref="B1:D26"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17.42578125" customWidth="1"/>
+    <col min="3" max="3" width="32.28515625" customWidth="1"/>
+    <col min="4" max="4" width="34.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:4" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:4" ht="41.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="3" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="D3" s="3" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="4" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B4" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>37</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="5" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B5" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="6" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B6" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="7" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B7" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="C7" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="8" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B8" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="9" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B9" s="4" t="s">
+        <v>51</v>
+      </c>
+      <c r="C9" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="10" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B10" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="11" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B11" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C11" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D11" s="3" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" spans="2:4" ht="114" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B12" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="15" spans="2:4" x14ac:dyDescent="0.25">
+      <c r="B15" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="2:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="B16" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="C16" s="6" t="s">
+        <v>64</v>
+      </c>
+      <c r="D16" s="6" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="17" spans="2:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="B17" s="7" t="s">
+        <v>82</v>
+      </c>
+      <c r="C17" s="6" t="s">
+        <v>66</v>
+      </c>
+      <c r="D17" s="6" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="18" spans="2:4" ht="90" x14ac:dyDescent="0.25">
+      <c r="B18" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="C18" s="6" t="s">
+        <v>67</v>
+      </c>
+      <c r="D18" s="6" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="19" spans="2:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="B19" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="C19" s="6" t="s">
+        <v>69</v>
+      </c>
+      <c r="D19" s="6" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="20" spans="2:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="B20" s="7" t="s">
+        <v>45</v>
+      </c>
+      <c r="C20" s="6" t="s">
+        <v>70</v>
+      </c>
+      <c r="D20" s="6" t="s">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="21" spans="2:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="B21" s="7" t="s">
+        <v>48</v>
+      </c>
+      <c r="C21" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="22" spans="2:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="B22" s="7" t="s">
+        <v>51</v>
+      </c>
+      <c r="C22" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="23" spans="2:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="B23" s="7" t="s">
+        <v>54</v>
+      </c>
+      <c r="C23" s="6" t="s">
+        <v>74</v>
+      </c>
+      <c r="D23" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="24" spans="2:4" ht="75" x14ac:dyDescent="0.25">
+      <c r="B24" s="7" t="s">
+        <v>57</v>
+      </c>
+      <c r="C24" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="D24" s="6" t="s">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="25" spans="2:4" ht="60" x14ac:dyDescent="0.25">
+      <c r="B25" s="7" t="s">
+        <v>60</v>
+      </c>
+      <c r="C25" s="6" t="s">
+        <v>77</v>
+      </c>
+      <c r="D25" s="6" t="s">
+        <v>78</v>
+      </c>
+    </row>
+    <row r="26" spans="2:4" ht="105" x14ac:dyDescent="0.25">
+      <c r="B26" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C26" s="6" t="s">
+        <v>80</v>
+      </c>
+      <c r="D26" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>